<commit_message>
Banheiro: caderno técnico R2 com nicho centrado e cores CMYK
Nicho da P1 centrado na parede (137,5 a 1.137,5 mm): ocupa as 13 colunas
centrais e os dois lados caem nas juntas. Pranchas redesenhadas na paleta
do caderno de paginação (branco, amarelo, ciano, magenta). Totais de peças
e caixas inalterados; orçamento R2 com a referência ao caderno atualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q227KRZLpQukG4UmT3AyJG
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_Banheiro_R2.xlsx
+++ b/orcamento/Orcamento_Banheiro_R2.xlsx
@@ -596,7 +596,7 @@
     <t xml:space="preserve">Projeto</t>
   </si>
   <si>
-    <t xml:space="preserve">R47; paredes Bleu Nuit com detalhes Nuage e tampo Nuage 7,5 × 15,5 cm. Paginação R2 no caderno técnico R1.</t>
+    <t xml:space="preserve">R47; paredes Bleu Nuit com detalhes Nuage e tampo Nuage 7,5 × 15,5 cm. Paginação no caderno técnico R2 (nicho centrado na P1).</t>
   </si>
   <si>
     <t xml:space="preserve">Contagem</t>
@@ -2723,14 +2723,14 @@
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">SUM(Paredes!F5:F19)</f>
-        <v>16.9531</v>
+        <v>16.9538</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.1</v>
       </c>
       <c r="E5" s="11" t="n">
         <f aca="false">C5*(1+D5)</f>
-        <v>18.64841</v>
+        <v>18.64918</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>0.3</v>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">SUM(Paredes!E5:E15)</f>
-        <v>17.604</v>
+        <v>17.6047</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2938,10 +2938,10 @@
         <v>2353</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>2.5994</v>
+        <v>2.6001</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>2.5064</v>
+        <v>2.5071</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>0.093</v>

</xml_diff>